<commit_message>
add route ratings methodology pdf
</commit_message>
<xml_diff>
--- a/research/files/route_metrics.xlsx
+++ b/research/files/route_metrics.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -511,7 +511,17 @@
       <c r="A13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>How every number here is computed, and what its limits are: https://bccycletourism.ca/research/files/route_ratings_methodology.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>The research here uses AI assistance (Claude models, Anthropic) for data collection, analysis, and writing. Feel free to ask for more details if you are interested.</t>
         </is>

</xml_diff>